<commit_message>
feat(eval): single gold evaluation of fixed models (Phase 5d)
PRIMARY (IndoBERT spec_3class/none + star 1-2 OR model): complaint F1 0.922 [0.89, 0.95] vs star rating 0.822, +0.099 [+0.071, +0.129]; precision unchanged.

TF-IDF binary_3star_negative + rule (comparison): 0.940; PRIMARY -0.019 [-0.038, -0.001].

4-5 star complaints: same-scheme IndoBERT and TF-IDF catch 36% vs 37%.

Intra-annotator (50 blind relabels; B035/B047 labeled): kappa 0.80 3-class, 0.90 binary.

W&B summary run phase5-summary
</commit_message>
<xml_diff>
--- a/data/gold/relabel_blind.xlsx
+++ b/data/gold/relabel_blind.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ewallet-review-analysis\data\gold\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C128723A-1EF9-4565-953E-093184783771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E550E148-7AD7-4EE8-A648-F6C2294BEA54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="107">
   <si>
     <t>gold_id</t>
   </si>
@@ -1127,7 +1127,9 @@
       <c r="B36" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C36" s="2"/>
+      <c r="C36" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="D36" s="2"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1269,7 +1271,9 @@
       <c r="B48" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C48" s="2"/>
+      <c r="C48" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="D48" s="2"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>